<commit_message>
feat(mech): complete 36 mechanical/fire protection activities, 108 HTMLs, and excel sheet integration
</commit_message>
<xml_diff>
--- a/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/동탄트램_공종별_매뉴얼_하이퍼링크_목록.xlsx
+++ b/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/동탄트램_공종별_매뉴얼_하이퍼링크_목록.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="신호" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전기" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통신" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기계" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,41 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00047857"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -96,8 +130,14 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -119,11 +159,25 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -165,6 +219,39 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7787,4 +7874,854 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>동탄도시철도(트램) 기계설비·소방설비 엔지니어링 매뉴얼 링크 대장</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>순번</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>액티비티명 (Activity)</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>표준서 (Standard)</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>수행지침 (Guideline)</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>체크리스트 (Checklist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>설계 적정성 검토</t>
+        </is>
+      </c>
+      <c r="C3" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\1_설계 적정성 검토\표준서\1_설계 적정성 검토_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D3" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\1_설계 적정성 검토\수행지침\1_설계 적정성 검토_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E3" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\1_설계 적정성 검토\체크리스트\1_설계 적정성 검토_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>발주전략 KOM</t>
+        </is>
+      </c>
+      <c r="C4" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\2_발주전략 KOM\표준서\2_발주전략 KOM_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D4" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\2_발주전략 KOM\수행지침\2_발주전략 KOM_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E4" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\2_발주전략 KOM\체크리스트\2_발주전략 KOM_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>3D BIM 기계_소방 간섭 검토</t>
+        </is>
+      </c>
+      <c r="C5" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\3_3D BIM 기계_소방 간섭 검토\표준서\3_3D BIM 기계_소방 간섭 검토_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D5" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\3_3D BIM 기계_소방 간섭 검토\수행지침\3_3D BIM 기계_소방 간섭 검토_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E5" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\3_3D BIM 기계_소방 간섭 검토\체크리스트\3_3D BIM 기계_소방 간섭 검토_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>소방 및 환경 인허가</t>
+        </is>
+      </c>
+      <c r="C6" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\4_소방 및 환경 인허가\표준서\4_소방 및 환경 인허가_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D6" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\4_소방 및 환경 인허가\수행지침\4_소방 및 환경 인허가_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E6" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\4_소방 및 환경 인허가\체크리스트\4_소방 및 환경 인허가_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>장비 반입동선 및 야적장 계획</t>
+        </is>
+      </c>
+      <c r="C7" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\5_장비 반입동선 및 야적장 계획\표준서\5_장비 반입동선 및 야적장 계획_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\5_장비 반입동선 및 야적장 계획\수행지침\5_장비 반입동선 및 야적장 계획_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E7" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\5_장비 반입동선 및 야적장 계획\체크리스트\5_장비 반입동선 및 야적장 계획_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Big Room 인터페이스 회의</t>
+        </is>
+      </c>
+      <c r="C8" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\6_Big Room 인터페이스 회의\표준서\6_Big Room 인터페이스 회의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D8" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\6_Big Room 인터페이스 회의\수행지침\6_Big Room 인터페이스 회의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E8" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\6_Big Room 인터페이스 회의\체크리스트\6_Big Room 인터페이스 회의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>지하매설 기계배관 협의</t>
+        </is>
+      </c>
+      <c r="C9" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\7_지하매설 기계배관 협의\표준서\7_지하매설 기계배관 협의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D9" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\7_지하매설 기계배관 협의\수행지침\7_지하매설 기계배관 협의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E9" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\7_지하매설 기계배관 협의\체크리스트\7_지하매설 기계배관 협의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>기계설비 시공계획서 수립</t>
+        </is>
+      </c>
+      <c r="C10" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\8_기계설비 시공계획서 수립\표준서\8_기계설비 시공계획서 수립_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D10" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\8_기계설비 시공계획서 수립\수행지침\8_기계설비 시공계획서 수립_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E10" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\8_기계설비 시공계획서 수립\체크리스트\8_기계설비 시공계획서 수립_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>주요 기계_소방 기자재 검수</t>
+        </is>
+      </c>
+      <c r="C11" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\9_주요 기계_소방 기자재 검수\표준서\9_주요 기계_소방 기자재 검수_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D11" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\9_주요 기계_소방 기자재 검수\수행지침\9_주요 기계_소방 기자재 검수_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E11" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\9_주요 기계_소방 기자재 검수\체크리스트\9_주요 기계_소방 기자재 검수_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>방화구획 내화채움구조 시공</t>
+        </is>
+      </c>
+      <c r="C12" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\10_방화구획 내화채움구조 시공\표준서\10_방화구획 내화채움구조 시공_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D12" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\10_방화구획 내화채움구조 시공\수행지침\10_방화구획 내화채움구조 시공_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E12" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\10_방화구획 내화채움구조 시공\체크리스트\10_방화구획 내화채움구조 시공_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>선로전환기 배수공동구 연계</t>
+        </is>
+      </c>
+      <c r="C13" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\11_선로전환기 배수공동구 연계\표준서\11_선로전환기 배수공동구 연계_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D13" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\11_선로전환기 배수공동구 연계\수행지침\11_선로전환기 배수공동구 연계_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E13" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\11_선로전환기 배수공동구 연계\체크리스트\11_선로전환기 배수공동구 연계_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>소방 기계 전원 간선 연계</t>
+        </is>
+      </c>
+      <c r="C14" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\12_소방 기계 전원 간선 연계\표준서\12_소방 기계 전원 간선 연계_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D14" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\12_소방 기계 전원 간선 연계\수행지침\12_소방 기계 전원 간선 연계_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E14" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\12_소방 기계 전원 간선 연계\체크리스트\12_소방 기계 전원 간선 연계_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>저수조 사수방지 흡입배관</t>
+        </is>
+      </c>
+      <c r="C15" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\13_저수조 사수방지 흡입배관\표준서\13_저수조 사수방지 흡입배관_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\13_저수조 사수방지 흡입배관\수행지침\13_저수조 사수방지 흡입배관_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E15" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\13_저수조 사수방지 흡입배관\체크리스트\13_저수조 사수방지 흡입배관_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>지열 신재생에너지 배관 매설</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\14_지열 신재생에너지 배관 매설\표준서\14_지열 신재생에너지 배관 매설_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D16" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\14_지열 신재생에너지 배관 매설\수행지침\14_지열 신재생에너지 배관 매설_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\14_지열 신재생에너지 배관 매설\체크리스트\14_지열 신재생에너지 배관 매설_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>정거장_변전소 환기덕트 시공</t>
+        </is>
+      </c>
+      <c r="C17" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\15_정거장_변전소 환기덕트 시공\표준서\15_정거장_변전소 환기덕트 시공_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D17" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\15_정거장_변전소 환기덕트 시공\수행지침\15_정거장_변전소 환기덕트 시공_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E17" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\15_정거장_변전소 환기덕트 시공\체크리스트\15_정거장_변전소 환기덕트 시공_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>고내열(250℃) 제연팬_풍도</t>
+        </is>
+      </c>
+      <c r="C18" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\16_고내열(250℃) 제연팬_풍도\표준서\16_고내열(250℃) 제연팬_풍도_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D18" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\16_고내열(250℃) 제연팬_풍도\수행지침\16_고내열(250℃) 제연팬_풍도_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E18" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\16_고내열(250℃) 제연팬_풍도\체크리스트\16_고내열(250℃) 제연팬_풍도_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>검수고 국부 냉난방 가설</t>
+        </is>
+      </c>
+      <c r="C19" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\17_검수고 국부 냉난방 가설\표준서\17_검수고 국부 냉난방 가설_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D19" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\17_검수고 국부 냉난방 가설\수행지침\17_검수고 국부 냉난방 가설_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E19" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\17_검수고 국부 냉난방 가설\체크리스트\17_검수고 국부 냉난방 가설_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>냉온수_냉각수 배관 용접</t>
+        </is>
+      </c>
+      <c r="C20" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\18_냉온수_냉각수 배관 용접\표준서\18_냉온수_냉각수 배관 용접_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D20" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\18_냉온수_냉각수 배관 용접\수행지침\18_냉온수_냉각수 배관 용접_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E20" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\18_냉온수_냉각수 배관 용접\체크리스트\18_냉온수_냉각수 배관 용접_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>능동지하차도 전용터널 제연</t>
+        </is>
+      </c>
+      <c r="C21" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\19_능동지하차도 전용터널 제연\표준서\19_능동지하차도 전용터널 제연_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\19_능동지하차도 전용터널 제연\수행지침\19_능동지하차도 전용터널 제연_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E21" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\19_능동지하차도 전용터널 제연\체크리스트\19_능동지하차도 전용터널 제연_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>공기조화기(AHU_PAC) 거치</t>
+        </is>
+      </c>
+      <c r="C22" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\20_공기조화기(AHU_PAC) 거치\표준서\20_공기조화기(AHU_PAC) 거치_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D22" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\20_공기조화기(AHU_PAC) 거치\수행지침\20_공기조화기(AHU_PAC) 거치_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E22" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\20_공기조화기(AHU_PAC) 거치\체크리스트\20_공기조화기(AHU_PAC) 거치_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>급수_급탕 STS 배관 시공</t>
+        </is>
+      </c>
+      <c r="C23" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\21_급수_급탕 STS 배관 시공\표준서\21_급수_급탕 STS 배관 시공_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\21_급수_급탕 STS 배관 시공\수행지침\21_급수_급탕 STS 배관 시공_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E23" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\21_급수_급탕 STS 배관 시공\체크리스트\21_급수_급탕 STS 배관 시공_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>오배수관 및 집수조 배수펌프</t>
+        </is>
+      </c>
+      <c r="C24" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\22_오배수관 및 집수조 배수펌프\표준서\22_오배수관 및 집수조 배수펌프_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D24" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\22_오배수관 및 집수조 배수펌프\수행지침\22_오배수관 및 집수조 배수펌프_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E24" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\22_오배수관 및 집수조 배수펌프\체크리스트\22_오배수관 및 집수조 배수펌프_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>차량기지 오폐수처리장(90㎡)</t>
+        </is>
+      </c>
+      <c r="C25" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\23_차량기지 오폐수처리장(90㎡)\표준서\23_차량기지 오폐수처리장(90㎡)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\23_차량기지 오폐수처리장(90㎡)\수행지침\23_차량기지 오폐수처리장(90㎡)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E25" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\23_차량기지 오폐수처리장(90㎡)\체크리스트\23_차량기지 오폐수처리장(90㎡)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>차체 자동세척설비(세차기)</t>
+        </is>
+      </c>
+      <c r="C26" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\24_차체 자동세척설비(세차기)\표준서\24_차체 자동세척설비(세차기)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D26" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\24_차체 자동세척설비(세차기)\수행지침\24_차체 자동세척설비(세차기)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E26" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\24_차체 자동세척설비(세차기)\체크리스트\24_차체 자동세척설비(세차기)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>정화조 음압 탈취설비 시공</t>
+        </is>
+      </c>
+      <c r="C27" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\25_정화조 음압 탈취설비 시공\표준서\25_정화조 음압 탈취설비 시공_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D27" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\25_정화조 음압 탈취설비 시공\수행지침\25_정화조 음압 탈취설비 시공_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E27" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\25_정화조 음압 탈취설비 시공\체크리스트\25_정화조 음압 탈취설비 시공_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="21" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>호스릴 옥내소화전설비 시공</t>
+        </is>
+      </c>
+      <c r="C28" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\26_호스릴 옥내소화전설비 시공\표준서\26_호스릴 옥내소화전설비 시공_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D28" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\26_호스릴 옥내소화전설비 시공\수행지침\26_호스릴 옥내소화전설비 시공_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E28" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\26_호스릴 옥내소화전설비 시공\체크리스트\26_호스릴 옥내소화전설비 시공_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>연결송수관-스프링클러 주배관 분리</t>
+        </is>
+      </c>
+      <c r="C29" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\27_연결송수관-스프링클러 주배관 분리\표준서\27_연결송수관-스프링클러 주배관 분리_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\27_연결송수관-스프링클러 주배관 분리\수행지침\27_연결송수관-스프링클러 주배관 분리_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E29" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\27_연결송수관-스프링클러 주배관 분리\체크리스트\27_연결송수관-스프링클러 주배관 분리_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="21" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>큐비클 가스계_에어로졸 소화</t>
+        </is>
+      </c>
+      <c r="C30" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\28_큐비클 가스계_에어로졸 소화\표준서\28_큐비클 가스계_에어로졸 소화_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D30" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\28_큐비클 가스계_에어로졸 소화\수행지침\28_큐비클 가스계_에어로졸 소화_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E30" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\28_큐비클 가스계_에어로졸 소화\체크리스트\28_큐비클 가스계_에어로졸 소화_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>가스소화구역 과압배출구(P.R.D)</t>
+        </is>
+      </c>
+      <c r="C31" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\29_가스소화구역 과압배출구(P.R.D)\표준서\29_가스소화구역 과압배출구(P.R.D)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\29_가스소화구역 과압배출구(P.R.D)\수행지침\29_가스소화구역 과압배출구(P.R.D)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E31" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\29_가스소화구역 과압배출구(P.R.D)\체크리스트\29_가스소화구역 과압배출구(P.R.D)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>소방펌프실 가설 및 성능시험</t>
+        </is>
+      </c>
+      <c r="C32" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\30_소방펌프실 가설 및 성능시험\표준서\30_소방펌프실 가설 및 성능시험_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D32" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\30_소방펌프실 가설 및 성능시험\수행지침\30_소방펌프실 가설 및 성능시험_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E32" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\30_소방펌프실 가설 및 성능시험\체크리스트\30_소방펌프실 가설 및 성능시험_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>정거장 인승용 승강기(17_24인승)</t>
+        </is>
+      </c>
+      <c r="C33" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\31_정거장 인승용 승강기(17_24인승)\표준서\31_정거장 인승용 승강기(17_24인승)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\31_정거장 인승용 승강기(17_24인승)\수행지침\31_정거장 인승용 승강기(17_24인승)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E33" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\31_정거장 인승용 승강기(17_24인승)\체크리스트\31_정거장 인승용 승강기(17_24인승)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>검수고 관통형 화물용 EV</t>
+        </is>
+      </c>
+      <c r="C34" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\32_검수고 관통형 화물용 EV\표준서\32_검수고 관통형 화물용 EV_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D34" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\32_검수고 관통형 화물용 EV\수행지침\32_검수고 관통형 화물용 EV_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E34" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\32_검수고 관통형 화물용 EV\체크리스트\32_검수고 관통형 화물용 EV_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>DDC_IP DDC 자동제어 백업 이중화</t>
+        </is>
+      </c>
+      <c r="C35" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\33_DDC_IP DDC 자동제어 백업 이중화\표준서\33_DDC_IP DDC 자동제어 백업 이중화_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D35" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\33_DDC_IP DDC 자동제어 백업 이중화\수행지침\33_DDC_IP DDC 자동제어 백업 이중화_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E35" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\33_DDC_IP DDC 자동제어 백업 이중화\체크리스트\33_DDC_IP DDC 자동제어 백업 이중화_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="21" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>화재연동 인터록 실부하 시험</t>
+        </is>
+      </c>
+      <c r="C36" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\34_화재연동 인터록 실부하 시험\표준서\34_화재연동 인터록 실부하 시험_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D36" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\34_화재연동 인터록 실부하 시험\수행지침\34_화재연동 인터록 실부하 시험_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E36" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\34_화재연동 인터록 실부하 시험\체크리스트\34_화재연동 인터록 실부하 시험_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>TAB(풍량_수량 밸런싱) 측정</t>
+        </is>
+      </c>
+      <c r="C37" s="18">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\35_TAB(풍량_수량 밸런싱) 측정\표준서\35_TAB(풍량_수량 밸런싱) 측정_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\35_TAB(풍량_수량 밸런싱) 측정\수행지침\35_TAB(풍량_수량 밸런싱) 측정_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E37" s="20">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\35_TAB(풍량_수량 밸런싱) 측정\체크리스트\35_TAB(풍량_수량 밸런싱) 측정_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="21" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>소방 완공검사 및 종합인계</t>
+        </is>
+      </c>
+      <c r="C38" s="23">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\36_소방 완공검사 및 종합인계\표준서\36_소방 완공검사 및 종합인계_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D38" s="24">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\36_소방 완공검사 및 종합인계\수행지침\36_소방 완공검사 및 종합인계_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E38" s="25">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\10.기계분야\36_소방 완공검사 및 종합인계\체크리스트\36_소방 완공검사 및 종합인계_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(commissioning): complete 28 commissioning activities, 84 HTMLs, and excel sheet integration based on KYH manual
</commit_message>
<xml_diff>
--- a/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/동탄트램_공종별_매뉴얼_하이퍼링크_목록.xlsx
+++ b/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/동탄트램_공종별_매뉴얼_하이퍼링크_목록.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전기" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통신" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기계" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="철도종합시운전" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -244,6 +245,33 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1463,6 +1491,680 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>동탄도시철도(트램) 철도종합시운전 엔지니어링 매뉴얼 링크 대장</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>순번</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>액티비티명 (Activity)</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>표준서 (Standard)</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>수행지침 (Guideline)</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>체크리스트 (Checklist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 사전검토</t>
+        </is>
+      </c>
+      <c r="C3" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\1_철도종합시험운행 사전검토\표준서\1_철도종합시험운행 사전검토_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D3" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\1_철도종합시험운행 사전검토\수행지침\1_철도종합시험운행 사전검토_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E3" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\1_철도종합시험운행 사전검토\체크리스트\1_철도종합시험운행 사전검토_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 사전검토 회의</t>
+        </is>
+      </c>
+      <c r="C4" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\2_철도종합시험운행 사전검토 회의\표준서\2_철도종합시험운행 사전검토 회의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D4" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\2_철도종합시험운행 사전검토 회의\수행지침\2_철도종합시험운행 사전검토 회의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E4" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\2_철도종합시험운행 사전검토 회의\체크리스트\2_철도종합시험운행 사전검토 회의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>토목·궤도 인터페이스 협의</t>
+        </is>
+      </c>
+      <c r="C5" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\3_토목·궤도 인터페이스 협의\표준서\3_토목·궤도 인터페이스 협의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D5" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\3_토목·궤도 인터페이스 협의\수행지침\3_토목·궤도 인터페이스 협의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E5" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\3_토목·궤도 인터페이스 협의\체크리스트\3_토목·궤도 인터페이스 협의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>전기·통신·신호·차량 인터페이스 협의</t>
+        </is>
+      </c>
+      <c r="C6" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\4_전기·통신·신호·차량 인터페이스 협의\표준서\4_전기·통신·신호·차량 인터페이스 협의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D6" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\4_전기·통신·신호·차량 인터페이스 협의\수행지침\4_전기·통신·신호·차량 인터페이스 협의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E6" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\4_전기·통신·신호·차량 인터페이스 협의\체크리스트\4_전기·통신·신호·차량 인터페이스 협의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>관제 및 운영사 인터페이스 협의</t>
+        </is>
+      </c>
+      <c r="C7" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\5_관제 및 운영사 인터페이스 협의\표준서\5_관제 및 운영사 인터페이스 협의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D7" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\5_관제 및 운영사 인터페이스 협의\수행지침\5_관제 및 운영사 인터페이스 협의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E7" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\5_관제 및 운영사 인터페이스 협의\체크리스트\5_관제 및 운영사 인터페이스 협의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>인력·시험장비 투입계획 수립</t>
+        </is>
+      </c>
+      <c r="C8" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\6_인력·시험장비 투입계획 수립\표준서\6_인력·시험장비 투입계획 수립_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D8" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\6_인력·시험장비 투입계획 수립\수행지침\6_인력·시험장비 투입계획 수립_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\6_인력·시험장비 투입계획 수립\체크리스트\6_인력·시험장비 투입계획 수립_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 사전 협의사항(TS) 도출</t>
+        </is>
+      </c>
+      <c r="C9" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\7_철도종합시험운행 사전 협의사항(TS) 도출\표준서\7_철도종합시험운행 사전 협의사항(TS) 도출_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D9" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\7_철도종합시험운행 사전 협의사항(TS) 도출\수행지침\7_철도종합시험운행 사전 협의사항(TS) 도출_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E9" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\7_철도종합시험운행 사전 협의사항(TS) 도출\체크리스트\7_철도종합시험운행 사전 협의사항(TS) 도출_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>착수 전 전공종 합동회의</t>
+        </is>
+      </c>
+      <c r="C10" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증\표준서\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D10" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증\수행지침\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E10" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증\체크리스트\8_착수 전 전공종 합동회의 및 공종별시험 완료 검증_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 종합계획서 수립</t>
+        </is>
+      </c>
+      <c r="C11" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\9_철도종합시험운행 종합계획서(SOP) 수립\표준서\9_철도종합시험운행 종합계획서(SOP) 수립_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D11" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\9_철도종합시험운행 종합계획서(SOP) 수립\수행지침\9_철도종합시험운행 종합계획서(SOP) 수립_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E11" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\9_철도종합시험운행 종합계획서(SOP) 수립\체크리스트\9_철도종합시험운행 종합계획서(SOP) 수립_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>TS 사전컨설팅 회의</t>
+        </is>
+      </c>
+      <c r="C12" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\10_계획서 제출 전 TS 사전컨설팅 회의\표준서\10_계획서 제출 전 TS 사전컨설팅 회의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\10_계획서 제출 전 TS 사전컨설팅 회의\수행지침\10_계획서 제출 전 TS 사전컨설팅 회의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E12" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\10_계획서 제출 전 TS 사전컨설팅 회의\체크리스트\10_계획서 제출 전 TS 사전컨설팅 회의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 연간계획 수립/제출</t>
+        </is>
+      </c>
+      <c r="C13" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\11_철도종합시험운행 연간계획 수립 및 TS 제출\표준서\11_철도종합시험운행 연간계획 수립 및 TS 제출_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D13" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\11_철도종합시험운행 연간계획 수립 및 TS 제출\수행지침\11_철도종합시험운행 연간계획 수립 및 TS 제출_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E13" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\11_철도종합시험운행 연간계획 수립 및 TS 제출\체크리스트\11_철도종합시험운행 연간계획 수립 및 TS 제출_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>안전관리계획서 수립 및 비상대응체계</t>
+        </is>
+      </c>
+      <c r="C14" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\12_시험운행 안전관리계획서 수립 및 비상대응체계\표준서\12_시험운행 안전관리계획서 수립 및 비상대응체계_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D14" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\12_시험운행 안전관리계획서 수립 및 비상대응체계\수행지침\12_시험운행 안전관리계획서 수립 및 비상대응체계_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E14" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\12_시험운행 안전관리계획서 수립 및 비상대응체계\체크리스트\12_시험운행 안전관리계획서 수립 및 비상대응체계_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>사전점검 착수보고</t>
+        </is>
+      </c>
+      <c r="C15" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\13_사전점검 착수보고 및 분야별 점검단 가동\표준서\13_사전점검 착수보고 및 분야별 점검단 가동_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D15" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\13_사전점검 착수보고 및 분야별 점검단 가동\수행지침\13_사전점검 착수보고 및 분야별 점검단 가동_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E15" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\13_사전점검 착수보고 및 분야별 점검단 가동\체크리스트\13_사전점검 착수보고 및 분야별 점검단 가동_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="31" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>철도시설 기술기준 검토 및 조치계획</t>
+        </is>
+      </c>
+      <c r="C16" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\14_철도시설의 기술기준 검토 및 지적사항 조치계획\표준서\14_철도시설의 기술기준 검토 및 지적사항 조치계획_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D16" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\14_철도시설의 기술기준 검토 및 지적사항 조치계획\수행지침\14_철도시설의 기술기준 검토 및 지적사항 조치계획_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E16" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\14_철도시설의 기술기준 검토 및 지적사항 조치계획\체크리스트\14_철도시설의 기술기준 검토 및 지적사항 조치계획_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>사전점검 보완조치 및 국토부 승인</t>
+        </is>
+      </c>
+      <c r="C17" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\15_사전점검 보완조치 및 조치결과 국토부 승인\표준서\15_사전점검 보완조치 및 조치결과 국토부 승인_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D17" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\15_사전점검 보완조치 및 조치결과 국토부 승인\수행지침\15_사전점검 보완조치 및 조치결과 국토부 승인_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E17" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\15_사전점검 보완조치 및 조치결과 국토부 승인\체크리스트\15_사전점검 보완조치 및 조치결과 국토부 승인_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>사전점검 종결회의 및 결과보고서 승인</t>
+        </is>
+      </c>
+      <c r="C18" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\16_사전점검 종결회의 및 결과보고서 승인\표준서\16_사전점검 종결회의 및 결과보고서 승인_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D18" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\16_사전점검 종결회의 및 결과보고서 승인\수행지침\16_사전점검 종결회의 및 결과보고서 승인_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E18" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\16_사전점검 종결회의 및 결과보고서 승인\체크리스트\16_사전점검 종결회의 및 결과보고서 승인_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>시설물검증시험 착수보고 및 안전교육</t>
+        </is>
+      </c>
+      <c r="C19" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\17_시설물검증시험 착수보고 및 시험참여자 안전교육\표준서\17_시설물검증시험 착수보고 및 시험참여자 안전교육_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D19" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\17_시설물검증시험 착수보고 및 시험참여자 안전교육\수행지침\17_시설물검증시험 착수보고 및 시험참여자 안전교육_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E19" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\17_시설물검증시험 착수보고 및 시험참여자 안전교육\체크리스트\17_시설물검증시험 착수보고 및 시험참여자 안전교육_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="31" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>시험열차 투입 및 속도별 연동시험</t>
+        </is>
+      </c>
+      <c r="C20" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\18_시험열차 투입계획 및 본선 속도별 연동 주행시험\표준서\18_시험열차 투입계획 및 본선 속도별 연동 주행시험_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D20" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\18_시험열차 투입계획 및 본선 속도별 연동 주행시험\수행지침\18_시험열차 투입계획 및 본선 속도별 연동 주행시험_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E20" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\18_시험열차 투입계획 및 본선 속도별 연동 주행시험\체크리스트\18_시험열차 투입계획 및 본선 속도별 연동 주행시험_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="27" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>시설물검증시험 중간점검 및 장애조치</t>
+        </is>
+      </c>
+      <c r="C21" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\19_시설물검증시험 중간점검 및 장애조치 회의\표준서\19_시설물검증시험 중간점검 및 장애조치 회의_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D21" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\19_시설물검증시험 중간점검 및 장애조치 회의\수행지침\19_시설물검증시험 중간점검 및 장애조치 회의_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E21" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\19_시설물검증시험 중간점검 및 장애조치 회의\체크리스트\19_시설물검증시험 중간점검 및 장애조치 회의_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>시설물검증시험 종결회의 및 결과 승인</t>
+        </is>
+      </c>
+      <c r="C22" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\20_시설물검증시험 종결회의 및 결과보고서 획득\표준서\20_시설물검증시험 종결회의 및 결과보고서 획득_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D22" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\20_시설물검증시험 종결회의 및 결과보고서 획득\수행지침\20_시설물검증시험 종결회의 및 결과보고서 획득_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E22" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\20_시설물검증시험 종결회의 및 결과보고서 획득\체크리스트\20_시설물검증시험 종결회의 및 결과보고서 획득_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="27" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>영업시운전 계획 수립 및 착수보고</t>
+        </is>
+      </c>
+      <c r="C23" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\21_영업시운전 계획 수립 및 착수보고(TS)\표준서\21_영업시운전 계획 수립 및 착수보고(TS)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D23" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\21_영업시운전 계획 수립 및 착수보고(TS)\수행지침\21_영업시운전 계획 수립 및 착수보고(TS)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E23" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\21_영업시운전 계획 수립 및 착수보고(TS)\체크리스트\21_영업시운전 계획 수립 및 착수보고(TS)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="31" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>영업 다이아 운행 및 비상대응훈련</t>
+        </is>
+      </c>
+      <c r="C24" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련\표준서\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D24" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련\수행지침\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E24" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련\체크리스트\22_실제 열차운행 다이아 기반 영업시운전 및 비상훈련_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>영업시운전 중간점검 및 조치</t>
+        </is>
+      </c>
+      <c r="C25" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\23_영업시운전 중간점검 및 이례상황 조치결과 검토\표준서\23_영업시운전 중간점검 및 이례상황 조치결과 검토_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D25" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\23_영업시운전 중간점검 및 이례상황 조치결과 검토\수행지침\23_영업시운전 중간점검 및 이례상황 조치결과 검토_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E25" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\23_영업시운전 중간점검 및 이례상황 조치결과 검토\체크리스트\23_영업시운전 중간점검 및 이례상황 조치결과 검토_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>영업시운전 종결회의 및 결과보고서 승인</t>
+        </is>
+      </c>
+      <c r="C26" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\24_영업시운전 종결회의 및 결과보고서 승인\표준서\24_영업시운전 종결회의 및 결과보고서 승인_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D26" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\24_영업시운전 종결회의 및 결과보고서 승인\수행지침\24_영업시운전 종결회의 및 결과보고서 승인_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E26" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\24_영업시운전 종결회의 및 결과보고서 승인\체크리스트\24_영업시운전 종결회의 및 결과보고서 승인_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>철도종합시험운행 종합결과보고서 제출</t>
+        </is>
+      </c>
+      <c r="C27" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\25_철도종합시험운행 종합결과보고서 작성 및 제출\표준서\25_철도종합시험운행 종합결과보고서 작성 및 제출_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D27" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\25_철도종합시험운행 종합결과보고서 작성 및 제출\수행지침\25_철도종합시험운행 종합결과보고서 작성 및 제출_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E27" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\25_철도종합시험운행 종합결과보고서 작성 및 제출\체크리스트\25_철도종합시험운행 종합결과보고서 작성 및 제출_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="31" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>철도운영자 안전관리체계 변경승인</t>
+        </is>
+      </c>
+      <c r="C28" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\26_철도운영자 안전관리체계 변경승인(TS)\표준서\26_철도운영자 안전관리체계 변경승인(TS)_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D28" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\26_철도운영자 안전관리체계 변경승인(TS)\수행지침\26_철도운영자 안전관리체계 변경승인(TS)_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E28" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\26_철도운영자 안전관리체계 변경승인(TS)\체크리스트\26_철도운영자 안전관리체계 변경승인(TS)_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>공사목적물 및 시설물 최종 인수인계</t>
+        </is>
+      </c>
+      <c r="C29" s="28">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\27_공사목적물 및 시설물 운영사 최종 인수인계\표준서\27_공사목적물 및 시설물 운영사 최종 인수인계_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D29" s="29">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\27_공사목적물 및 시설물 운영사 최종 인수인계\수행지침\27_공사목적물 및 시설물 운영사 최종 인수인계_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E29" s="30">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\27_공사목적물 및 시설물 운영사 최종 인수인계\체크리스트\27_공사목적물 및 시설물 운영사 최종 인수인계_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>종합시험운행 종결 및 영업 개통</t>
+        </is>
+      </c>
+      <c r="C30" s="32">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통\표준서\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통_표준서.html", "📄 표준서 열기")</f>
+        <v/>
+      </c>
+      <c r="D30" s="33">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통\수행지침\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통_수행지침.html", "📘 수행지침 열기")</f>
+        <v/>
+      </c>
+      <c r="E30" s="34">
+        <f>HYPERLINK(LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"매뉴얼BODY(집행단계-첨부폴더)v8\11.철도종합시운전\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통\체크리스트\28_동탄도시철도(트램) 종합시험운행 종결 및 영업 개통_체크리스트.html", "📋 체크리스트 열기")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>